<commit_message>
Fix workbook errors: Settings formula text, column widths, empty row guards
- Settings D8/D9: Remove leading '=' from help text that caused Err:509
- Home Loan Calc & Vehicle Loan Calc: Widen column D from 5 to 18 (was showing ###)
- Debt Tracker: Add empty-row guard to Interest Rate formula (was showing 11.25% for blank rows)
- Savings Tracker: Add empty-row guard to % of Goal, Remaining, Months to Goal
- Investments: Add empty-row guard to Gain/Loss and Gain/Loss % columns

All formula cells now show blank when the row has no data entered.

Co-Authored-By: Devin AI <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Personal_Finance_Workbook.xlsx
+++ b/Personal_Finance_Workbook.xlsx
@@ -1665,9 +1665,10 @@
         <f>C4+C5</f>
         <v/>
       </c>
-      <c r="D8" s="27">
-        <f> Prime + Home Loan Margin</f>
-        <v/>
+      <c r="D8" s="27" t="inlineStr">
+        <is>
+          <t>Prime + Home Loan Margin</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -1680,9 +1681,10 @@
         <f>C4+C6</f>
         <v/>
       </c>
-      <c r="D9" s="27">
-        <f> Prime + Vehicle Loan Margin</f>
-        <v/>
+      <c r="D9" s="27" t="inlineStr">
+        <is>
+          <t>Prime + Vehicle Loan Margin</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -3656,21 +3658,21 @@
       <c r="F5" s="17" t="n"/>
       <c r="G5" s="25" t="n"/>
       <c r="H5" s="22">
-        <f>IF(F5="Manual",G5,Settings!$C$4+G5)</f>
+        <f>IF(A5="","",IF(F5="Manual",G5,Settings!$C$4+G5))</f>
         <v/>
       </c>
       <c r="I5" s="15" t="n"/>
       <c r="J5" s="17" t="n"/>
       <c r="K5" s="20">
-        <f>IF(E5=0,0,E5*H5/12)</f>
+        <f>IF(A5="","",IF(E5=0,0,E5*H5/12))</f>
         <v/>
       </c>
       <c r="L5" s="20">
-        <f>IF(J5=0,0,K5*J5)</f>
+        <f>IF(A5="","",IF(J5=0,0,K5*J5))</f>
         <v/>
       </c>
       <c r="M5" s="22">
-        <f>IF(D5=0,0,1-(E5/D5))</f>
+        <f>IF(A5="","",IF(D5=0,0,1-(E5/D5)))</f>
         <v/>
       </c>
     </row>
@@ -3683,21 +3685,21 @@
       <c r="F6" s="17" t="n"/>
       <c r="G6" s="25" t="n"/>
       <c r="H6" s="22">
-        <f>IF(F6="Manual",G6,Settings!$C$4+G6)</f>
+        <f>IF(A6="","",IF(F6="Manual",G6,Settings!$C$4+G6))</f>
         <v/>
       </c>
       <c r="I6" s="15" t="n"/>
       <c r="J6" s="17" t="n"/>
       <c r="K6" s="20">
-        <f>IF(E6=0,0,E6*H6/12)</f>
+        <f>IF(A6="","",IF(E6=0,0,E6*H6/12))</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>IF(J6=0,0,K6*J6)</f>
+        <f>IF(A6="","",IF(J6=0,0,K6*J6))</f>
         <v/>
       </c>
       <c r="M6" s="22">
-        <f>IF(D6=0,0,1-(E6/D6))</f>
+        <f>IF(A6="","",IF(D6=0,0,1-(E6/D6)))</f>
         <v/>
       </c>
     </row>
@@ -3710,21 +3712,21 @@
       <c r="F7" s="17" t="n"/>
       <c r="G7" s="25" t="n"/>
       <c r="H7" s="22">
-        <f>IF(F7="Manual",G7,Settings!$C$4+G7)</f>
+        <f>IF(A7="","",IF(F7="Manual",G7,Settings!$C$4+G7))</f>
         <v/>
       </c>
       <c r="I7" s="15" t="n"/>
       <c r="J7" s="17" t="n"/>
       <c r="K7" s="20">
-        <f>IF(E7=0,0,E7*H7/12)</f>
+        <f>IF(A7="","",IF(E7=0,0,E7*H7/12))</f>
         <v/>
       </c>
       <c r="L7" s="20">
-        <f>IF(J7=0,0,K7*J7)</f>
+        <f>IF(A7="","",IF(J7=0,0,K7*J7))</f>
         <v/>
       </c>
       <c r="M7" s="22">
-        <f>IF(D7=0,0,1-(E7/D7))</f>
+        <f>IF(A7="","",IF(D7=0,0,1-(E7/D7)))</f>
         <v/>
       </c>
     </row>
@@ -3737,21 +3739,21 @@
       <c r="F8" s="17" t="n"/>
       <c r="G8" s="25" t="n"/>
       <c r="H8" s="22">
-        <f>IF(F8="Manual",G8,Settings!$C$4+G8)</f>
+        <f>IF(A8="","",IF(F8="Manual",G8,Settings!$C$4+G8))</f>
         <v/>
       </c>
       <c r="I8" s="15" t="n"/>
       <c r="J8" s="17" t="n"/>
       <c r="K8" s="20">
-        <f>IF(E8=0,0,E8*H8/12)</f>
+        <f>IF(A8="","",IF(E8=0,0,E8*H8/12))</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>IF(J8=0,0,K8*J8)</f>
+        <f>IF(A8="","",IF(J8=0,0,K8*J8))</f>
         <v/>
       </c>
       <c r="M8" s="22">
-        <f>IF(D8=0,0,1-(E8/D8))</f>
+        <f>IF(A8="","",IF(D8=0,0,1-(E8/D8)))</f>
         <v/>
       </c>
     </row>
@@ -3764,21 +3766,21 @@
       <c r="F9" s="17" t="n"/>
       <c r="G9" s="25" t="n"/>
       <c r="H9" s="22">
-        <f>IF(F9="Manual",G9,Settings!$C$4+G9)</f>
+        <f>IF(A9="","",IF(F9="Manual",G9,Settings!$C$4+G9))</f>
         <v/>
       </c>
       <c r="I9" s="15" t="n"/>
       <c r="J9" s="17" t="n"/>
       <c r="K9" s="20">
-        <f>IF(E9=0,0,E9*H9/12)</f>
+        <f>IF(A9="","",IF(E9=0,0,E9*H9/12))</f>
         <v/>
       </c>
       <c r="L9" s="20">
-        <f>IF(J9=0,0,K9*J9)</f>
+        <f>IF(A9="","",IF(J9=0,0,K9*J9))</f>
         <v/>
       </c>
       <c r="M9" s="22">
-        <f>IF(D9=0,0,1-(E9/D9))</f>
+        <f>IF(A9="","",IF(D9=0,0,1-(E9/D9)))</f>
         <v/>
       </c>
     </row>
@@ -3791,21 +3793,21 @@
       <c r="F10" s="17" t="n"/>
       <c r="G10" s="25" t="n"/>
       <c r="H10" s="22">
-        <f>IF(F10="Manual",G10,Settings!$C$4+G10)</f>
+        <f>IF(A10="","",IF(F10="Manual",G10,Settings!$C$4+G10))</f>
         <v/>
       </c>
       <c r="I10" s="15" t="n"/>
       <c r="J10" s="17" t="n"/>
       <c r="K10" s="20">
-        <f>IF(E10=0,0,E10*H10/12)</f>
+        <f>IF(A10="","",IF(E10=0,0,E10*H10/12))</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>IF(J10=0,0,K10*J10)</f>
+        <f>IF(A10="","",IF(J10=0,0,K10*J10))</f>
         <v/>
       </c>
       <c r="M10" s="22">
-        <f>IF(D10=0,0,1-(E10/D10))</f>
+        <f>IF(A10="","",IF(D10=0,0,1-(E10/D10)))</f>
         <v/>
       </c>
     </row>
@@ -3818,21 +3820,21 @@
       <c r="F11" s="17" t="n"/>
       <c r="G11" s="25" t="n"/>
       <c r="H11" s="22">
-        <f>IF(F11="Manual",G11,Settings!$C$4+G11)</f>
+        <f>IF(A11="","",IF(F11="Manual",G11,Settings!$C$4+G11))</f>
         <v/>
       </c>
       <c r="I11" s="15" t="n"/>
       <c r="J11" s="17" t="n"/>
       <c r="K11" s="20">
-        <f>IF(E11=0,0,E11*H11/12)</f>
+        <f>IF(A11="","",IF(E11=0,0,E11*H11/12))</f>
         <v/>
       </c>
       <c r="L11" s="20">
-        <f>IF(J11=0,0,K11*J11)</f>
+        <f>IF(A11="","",IF(J11=0,0,K11*J11))</f>
         <v/>
       </c>
       <c r="M11" s="22">
-        <f>IF(D11=0,0,1-(E11/D11))</f>
+        <f>IF(A11="","",IF(D11=0,0,1-(E11/D11)))</f>
         <v/>
       </c>
     </row>
@@ -3845,21 +3847,21 @@
       <c r="F12" s="17" t="n"/>
       <c r="G12" s="25" t="n"/>
       <c r="H12" s="22">
-        <f>IF(F12="Manual",G12,Settings!$C$4+G12)</f>
+        <f>IF(A12="","",IF(F12="Manual",G12,Settings!$C$4+G12))</f>
         <v/>
       </c>
       <c r="I12" s="15" t="n"/>
       <c r="J12" s="17" t="n"/>
       <c r="K12" s="20">
-        <f>IF(E12=0,0,E12*H12/12)</f>
+        <f>IF(A12="","",IF(E12=0,0,E12*H12/12))</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>IF(J12=0,0,K12*J12)</f>
+        <f>IF(A12="","",IF(J12=0,0,K12*J12))</f>
         <v/>
       </c>
       <c r="M12" s="22">
-        <f>IF(D12=0,0,1-(E12/D12))</f>
+        <f>IF(A12="","",IF(D12=0,0,1-(E12/D12)))</f>
         <v/>
       </c>
     </row>
@@ -3872,21 +3874,21 @@
       <c r="F13" s="17" t="n"/>
       <c r="G13" s="25" t="n"/>
       <c r="H13" s="22">
-        <f>IF(F13="Manual",G13,Settings!$C$4+G13)</f>
+        <f>IF(A13="","",IF(F13="Manual",G13,Settings!$C$4+G13))</f>
         <v/>
       </c>
       <c r="I13" s="15" t="n"/>
       <c r="J13" s="17" t="n"/>
       <c r="K13" s="20">
-        <f>IF(E13=0,0,E13*H13/12)</f>
+        <f>IF(A13="","",IF(E13=0,0,E13*H13/12))</f>
         <v/>
       </c>
       <c r="L13" s="20">
-        <f>IF(J13=0,0,K13*J13)</f>
+        <f>IF(A13="","",IF(J13=0,0,K13*J13))</f>
         <v/>
       </c>
       <c r="M13" s="22">
-        <f>IF(D13=0,0,1-(E13/D13))</f>
+        <f>IF(A13="","",IF(D13=0,0,1-(E13/D13)))</f>
         <v/>
       </c>
     </row>
@@ -3899,21 +3901,21 @@
       <c r="F14" s="17" t="n"/>
       <c r="G14" s="25" t="n"/>
       <c r="H14" s="22">
-        <f>IF(F14="Manual",G14,Settings!$C$4+G14)</f>
+        <f>IF(A14="","",IF(F14="Manual",G14,Settings!$C$4+G14))</f>
         <v/>
       </c>
       <c r="I14" s="15" t="n"/>
       <c r="J14" s="17" t="n"/>
       <c r="K14" s="20">
-        <f>IF(E14=0,0,E14*H14/12)</f>
+        <f>IF(A14="","",IF(E14=0,0,E14*H14/12))</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>IF(J14=0,0,K14*J14)</f>
+        <f>IF(A14="","",IF(J14=0,0,K14*J14))</f>
         <v/>
       </c>
       <c r="M14" s="22">
-        <f>IF(D14=0,0,1-(E14/D14))</f>
+        <f>IF(A14="","",IF(D14=0,0,1-(E14/D14)))</f>
         <v/>
       </c>
     </row>
@@ -3926,21 +3928,21 @@
       <c r="F15" s="17" t="n"/>
       <c r="G15" s="25" t="n"/>
       <c r="H15" s="22">
-        <f>IF(F15="Manual",G15,Settings!$C$4+G15)</f>
+        <f>IF(A15="","",IF(F15="Manual",G15,Settings!$C$4+G15))</f>
         <v/>
       </c>
       <c r="I15" s="15" t="n"/>
       <c r="J15" s="17" t="n"/>
       <c r="K15" s="20">
-        <f>IF(E15=0,0,E15*H15/12)</f>
+        <f>IF(A15="","",IF(E15=0,0,E15*H15/12))</f>
         <v/>
       </c>
       <c r="L15" s="20">
-        <f>IF(J15=0,0,K15*J15)</f>
+        <f>IF(A15="","",IF(J15=0,0,K15*J15))</f>
         <v/>
       </c>
       <c r="M15" s="22">
-        <f>IF(D15=0,0,1-(E15/D15))</f>
+        <f>IF(A15="","",IF(D15=0,0,1-(E15/D15)))</f>
         <v/>
       </c>
     </row>
@@ -3953,21 +3955,21 @@
       <c r="F16" s="17" t="n"/>
       <c r="G16" s="25" t="n"/>
       <c r="H16" s="22">
-        <f>IF(F16="Manual",G16,Settings!$C$4+G16)</f>
+        <f>IF(A16="","",IF(F16="Manual",G16,Settings!$C$4+G16))</f>
         <v/>
       </c>
       <c r="I16" s="15" t="n"/>
       <c r="J16" s="17" t="n"/>
       <c r="K16" s="20">
-        <f>IF(E16=0,0,E16*H16/12)</f>
+        <f>IF(A16="","",IF(E16=0,0,E16*H16/12))</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>IF(J16=0,0,K16*J16)</f>
+        <f>IF(A16="","",IF(J16=0,0,K16*J16))</f>
         <v/>
       </c>
       <c r="M16" s="22">
-        <f>IF(D16=0,0,1-(E16/D16))</f>
+        <f>IF(A16="","",IF(D16=0,0,1-(E16/D16)))</f>
         <v/>
       </c>
     </row>
@@ -3980,21 +3982,21 @@
       <c r="F17" s="17" t="n"/>
       <c r="G17" s="25" t="n"/>
       <c r="H17" s="22">
-        <f>IF(F17="Manual",G17,Settings!$C$4+G17)</f>
+        <f>IF(A17="","",IF(F17="Manual",G17,Settings!$C$4+G17))</f>
         <v/>
       </c>
       <c r="I17" s="15" t="n"/>
       <c r="J17" s="17" t="n"/>
       <c r="K17" s="20">
-        <f>IF(E17=0,0,E17*H17/12)</f>
+        <f>IF(A17="","",IF(E17=0,0,E17*H17/12))</f>
         <v/>
       </c>
       <c r="L17" s="20">
-        <f>IF(J17=0,0,K17*J17)</f>
+        <f>IF(A17="","",IF(J17=0,0,K17*J17))</f>
         <v/>
       </c>
       <c r="M17" s="22">
-        <f>IF(D17=0,0,1-(E17/D17))</f>
+        <f>IF(A17="","",IF(D17=0,0,1-(E17/D17)))</f>
         <v/>
       </c>
     </row>
@@ -4007,21 +4009,21 @@
       <c r="F18" s="17" t="n"/>
       <c r="G18" s="25" t="n"/>
       <c r="H18" s="22">
-        <f>IF(F18="Manual",G18,Settings!$C$4+G18)</f>
+        <f>IF(A18="","",IF(F18="Manual",G18,Settings!$C$4+G18))</f>
         <v/>
       </c>
       <c r="I18" s="15" t="n"/>
       <c r="J18" s="17" t="n"/>
       <c r="K18" s="20">
-        <f>IF(E18=0,0,E18*H18/12)</f>
+        <f>IF(A18="","",IF(E18=0,0,E18*H18/12))</f>
         <v/>
       </c>
       <c r="L18" s="20">
-        <f>IF(J18=0,0,K18*J18)</f>
+        <f>IF(A18="","",IF(J18=0,0,K18*J18))</f>
         <v/>
       </c>
       <c r="M18" s="22">
-        <f>IF(D18=0,0,1-(E18/D18))</f>
+        <f>IF(A18="","",IF(D18=0,0,1-(E18/D18)))</f>
         <v/>
       </c>
     </row>
@@ -4034,21 +4036,21 @@
       <c r="F19" s="17" t="n"/>
       <c r="G19" s="25" t="n"/>
       <c r="H19" s="22">
-        <f>IF(F19="Manual",G19,Settings!$C$4+G19)</f>
+        <f>IF(A19="","",IF(F19="Manual",G19,Settings!$C$4+G19))</f>
         <v/>
       </c>
       <c r="I19" s="15" t="n"/>
       <c r="J19" s="17" t="n"/>
       <c r="K19" s="20">
-        <f>IF(E19=0,0,E19*H19/12)</f>
+        <f>IF(A19="","",IF(E19=0,0,E19*H19/12))</f>
         <v/>
       </c>
       <c r="L19" s="20">
-        <f>IF(J19=0,0,K19*J19)</f>
+        <f>IF(A19="","",IF(J19=0,0,K19*J19))</f>
         <v/>
       </c>
       <c r="M19" s="22">
-        <f>IF(D19=0,0,1-(E19/D19))</f>
+        <f>IF(A19="","",IF(D19=0,0,1-(E19/D19)))</f>
         <v/>
       </c>
     </row>
@@ -4061,21 +4063,21 @@
       <c r="F20" s="17" t="n"/>
       <c r="G20" s="25" t="n"/>
       <c r="H20" s="22">
-        <f>IF(F20="Manual",G20,Settings!$C$4+G20)</f>
+        <f>IF(A20="","",IF(F20="Manual",G20,Settings!$C$4+G20))</f>
         <v/>
       </c>
       <c r="I20" s="15" t="n"/>
       <c r="J20" s="17" t="n"/>
       <c r="K20" s="20">
-        <f>IF(E20=0,0,E20*H20/12)</f>
+        <f>IF(A20="","",IF(E20=0,0,E20*H20/12))</f>
         <v/>
       </c>
       <c r="L20" s="20">
-        <f>IF(J20=0,0,K20*J20)</f>
+        <f>IF(A20="","",IF(J20=0,0,K20*J20))</f>
         <v/>
       </c>
       <c r="M20" s="22">
-        <f>IF(D20=0,0,1-(E20/D20))</f>
+        <f>IF(A20="","",IF(D20=0,0,1-(E20/D20)))</f>
         <v/>
       </c>
     </row>
@@ -4088,21 +4090,21 @@
       <c r="F21" s="17" t="n"/>
       <c r="G21" s="25" t="n"/>
       <c r="H21" s="22">
-        <f>IF(F21="Manual",G21,Settings!$C$4+G21)</f>
+        <f>IF(A21="","",IF(F21="Manual",G21,Settings!$C$4+G21))</f>
         <v/>
       </c>
       <c r="I21" s="15" t="n"/>
       <c r="J21" s="17" t="n"/>
       <c r="K21" s="20">
-        <f>IF(E21=0,0,E21*H21/12)</f>
+        <f>IF(A21="","",IF(E21=0,0,E21*H21/12))</f>
         <v/>
       </c>
       <c r="L21" s="20">
-        <f>IF(J21=0,0,K21*J21)</f>
+        <f>IF(A21="","",IF(J21=0,0,K21*J21))</f>
         <v/>
       </c>
       <c r="M21" s="22">
-        <f>IF(D21=0,0,1-(E21/D21))</f>
+        <f>IF(A21="","",IF(D21=0,0,1-(E21/D21)))</f>
         <v/>
       </c>
     </row>
@@ -4115,21 +4117,21 @@
       <c r="F22" s="17" t="n"/>
       <c r="G22" s="25" t="n"/>
       <c r="H22" s="22">
-        <f>IF(F22="Manual",G22,Settings!$C$4+G22)</f>
+        <f>IF(A22="","",IF(F22="Manual",G22,Settings!$C$4+G22))</f>
         <v/>
       </c>
       <c r="I22" s="15" t="n"/>
       <c r="J22" s="17" t="n"/>
       <c r="K22" s="20">
-        <f>IF(E22=0,0,E22*H22/12)</f>
+        <f>IF(A22="","",IF(E22=0,0,E22*H22/12))</f>
         <v/>
       </c>
       <c r="L22" s="20">
-        <f>IF(J22=0,0,K22*J22)</f>
+        <f>IF(A22="","",IF(J22=0,0,K22*J22))</f>
         <v/>
       </c>
       <c r="M22" s="22">
-        <f>IF(D22=0,0,1-(E22/D22))</f>
+        <f>IF(A22="","",IF(D22=0,0,1-(E22/D22)))</f>
         <v/>
       </c>
     </row>
@@ -4142,21 +4144,21 @@
       <c r="F23" s="17" t="n"/>
       <c r="G23" s="25" t="n"/>
       <c r="H23" s="22">
-        <f>IF(F23="Manual",G23,Settings!$C$4+G23)</f>
+        <f>IF(A23="","",IF(F23="Manual",G23,Settings!$C$4+G23))</f>
         <v/>
       </c>
       <c r="I23" s="15" t="n"/>
       <c r="J23" s="17" t="n"/>
       <c r="K23" s="20">
-        <f>IF(E23=0,0,E23*H23/12)</f>
+        <f>IF(A23="","",IF(E23=0,0,E23*H23/12))</f>
         <v/>
       </c>
       <c r="L23" s="20">
-        <f>IF(J23=0,0,K23*J23)</f>
+        <f>IF(A23="","",IF(J23=0,0,K23*J23))</f>
         <v/>
       </c>
       <c r="M23" s="22">
-        <f>IF(D23=0,0,1-(E23/D23))</f>
+        <f>IF(A23="","",IF(D23=0,0,1-(E23/D23)))</f>
         <v/>
       </c>
     </row>
@@ -4169,21 +4171,21 @@
       <c r="F24" s="17" t="n"/>
       <c r="G24" s="25" t="n"/>
       <c r="H24" s="22">
-        <f>IF(F24="Manual",G24,Settings!$C$4+G24)</f>
+        <f>IF(A24="","",IF(F24="Manual",G24,Settings!$C$4+G24))</f>
         <v/>
       </c>
       <c r="I24" s="15" t="n"/>
       <c r="J24" s="17" t="n"/>
       <c r="K24" s="20">
-        <f>IF(E24=0,0,E24*H24/12)</f>
+        <f>IF(A24="","",IF(E24=0,0,E24*H24/12))</f>
         <v/>
       </c>
       <c r="L24" s="20">
-        <f>IF(J24=0,0,K24*J24)</f>
+        <f>IF(A24="","",IF(J24=0,0,K24*J24))</f>
         <v/>
       </c>
       <c r="M24" s="22">
-        <f>IF(D24=0,0,1-(E24/D24))</f>
+        <f>IF(A24="","",IF(D24=0,0,1-(E24/D24)))</f>
         <v/>
       </c>
     </row>
@@ -4272,7 +4274,7 @@
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="5" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
@@ -11996,7 +11998,7 @@
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="5" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
@@ -14157,15 +14159,15 @@
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="15" t="n"/>
       <c r="F5" s="22">
-        <f>IF(E5=0,0,MIN(1,C5/E5))</f>
+        <f>IF(A5="","",IF(E5=0,0,MIN(1,C5/E5)))</f>
         <v/>
       </c>
       <c r="G5" s="20">
-        <f>IF(E5=0,0,MAX(0,E5-C5))</f>
+        <f>IF(A5="","",IF(E5=0,0,MAX(0,E5-C5)))</f>
         <v/>
       </c>
       <c r="H5" s="31">
-        <f>IF(OR(D5=0,G5&lt;=0),"N/A",ROUNDUP(G5/D5,0))</f>
+        <f>IF(A5="","",IF(OR(D5=0,G5&lt;=0),"N/A",ROUNDUP(G5/D5,0)))</f>
         <v/>
       </c>
     </row>
@@ -14176,15 +14178,15 @@
       <c r="D6" s="15" t="n"/>
       <c r="E6" s="15" t="n"/>
       <c r="F6" s="22">
-        <f>IF(E6=0,0,MIN(1,C6/E6))</f>
+        <f>IF(A6="","",IF(E6=0,0,MIN(1,C6/E6)))</f>
         <v/>
       </c>
       <c r="G6" s="20">
-        <f>IF(E6=0,0,MAX(0,E6-C6))</f>
+        <f>IF(A6="","",IF(E6=0,0,MAX(0,E6-C6)))</f>
         <v/>
       </c>
       <c r="H6" s="31">
-        <f>IF(OR(D6=0,G6&lt;=0),"N/A",ROUNDUP(G6/D6,0))</f>
+        <f>IF(A6="","",IF(OR(D6=0,G6&lt;=0),"N/A",ROUNDUP(G6/D6,0)))</f>
         <v/>
       </c>
     </row>
@@ -14195,15 +14197,15 @@
       <c r="D7" s="15" t="n"/>
       <c r="E7" s="15" t="n"/>
       <c r="F7" s="22">
-        <f>IF(E7=0,0,MIN(1,C7/E7))</f>
+        <f>IF(A7="","",IF(E7=0,0,MIN(1,C7/E7)))</f>
         <v/>
       </c>
       <c r="G7" s="20">
-        <f>IF(E7=0,0,MAX(0,E7-C7))</f>
+        <f>IF(A7="","",IF(E7=0,0,MAX(0,E7-C7)))</f>
         <v/>
       </c>
       <c r="H7" s="31">
-        <f>IF(OR(D7=0,G7&lt;=0),"N/A",ROUNDUP(G7/D7,0))</f>
+        <f>IF(A7="","",IF(OR(D7=0,G7&lt;=0),"N/A",ROUNDUP(G7/D7,0)))</f>
         <v/>
       </c>
     </row>
@@ -14214,15 +14216,15 @@
       <c r="D8" s="15" t="n"/>
       <c r="E8" s="15" t="n"/>
       <c r="F8" s="22">
-        <f>IF(E8=0,0,MIN(1,C8/E8))</f>
+        <f>IF(A8="","",IF(E8=0,0,MIN(1,C8/E8)))</f>
         <v/>
       </c>
       <c r="G8" s="20">
-        <f>IF(E8=0,0,MAX(0,E8-C8))</f>
+        <f>IF(A8="","",IF(E8=0,0,MAX(0,E8-C8)))</f>
         <v/>
       </c>
       <c r="H8" s="31">
-        <f>IF(OR(D8=0,G8&lt;=0),"N/A",ROUNDUP(G8/D8,0))</f>
+        <f>IF(A8="","",IF(OR(D8=0,G8&lt;=0),"N/A",ROUNDUP(G8/D8,0)))</f>
         <v/>
       </c>
     </row>
@@ -14233,15 +14235,15 @@
       <c r="D9" s="15" t="n"/>
       <c r="E9" s="15" t="n"/>
       <c r="F9" s="22">
-        <f>IF(E9=0,0,MIN(1,C9/E9))</f>
+        <f>IF(A9="","",IF(E9=0,0,MIN(1,C9/E9)))</f>
         <v/>
       </c>
       <c r="G9" s="20">
-        <f>IF(E9=0,0,MAX(0,E9-C9))</f>
+        <f>IF(A9="","",IF(E9=0,0,MAX(0,E9-C9)))</f>
         <v/>
       </c>
       <c r="H9" s="31">
-        <f>IF(OR(D9=0,G9&lt;=0),"N/A",ROUNDUP(G9/D9,0))</f>
+        <f>IF(A9="","",IF(OR(D9=0,G9&lt;=0),"N/A",ROUNDUP(G9/D9,0)))</f>
         <v/>
       </c>
     </row>
@@ -14252,15 +14254,15 @@
       <c r="D10" s="15" t="n"/>
       <c r="E10" s="15" t="n"/>
       <c r="F10" s="22">
-        <f>IF(E10=0,0,MIN(1,C10/E10))</f>
+        <f>IF(A10="","",IF(E10=0,0,MIN(1,C10/E10)))</f>
         <v/>
       </c>
       <c r="G10" s="20">
-        <f>IF(E10=0,0,MAX(0,E10-C10))</f>
+        <f>IF(A10="","",IF(E10=0,0,MAX(0,E10-C10)))</f>
         <v/>
       </c>
       <c r="H10" s="31">
-        <f>IF(OR(D10=0,G10&lt;=0),"N/A",ROUNDUP(G10/D10,0))</f>
+        <f>IF(A10="","",IF(OR(D10=0,G10&lt;=0),"N/A",ROUNDUP(G10/D10,0)))</f>
         <v/>
       </c>
     </row>
@@ -14271,15 +14273,15 @@
       <c r="D11" s="15" t="n"/>
       <c r="E11" s="15" t="n"/>
       <c r="F11" s="22">
-        <f>IF(E11=0,0,MIN(1,C11/E11))</f>
+        <f>IF(A11="","",IF(E11=0,0,MIN(1,C11/E11)))</f>
         <v/>
       </c>
       <c r="G11" s="20">
-        <f>IF(E11=0,0,MAX(0,E11-C11))</f>
+        <f>IF(A11="","",IF(E11=0,0,MAX(0,E11-C11)))</f>
         <v/>
       </c>
       <c r="H11" s="31">
-        <f>IF(OR(D11=0,G11&lt;=0),"N/A",ROUNDUP(G11/D11,0))</f>
+        <f>IF(A11="","",IF(OR(D11=0,G11&lt;=0),"N/A",ROUNDUP(G11/D11,0)))</f>
         <v/>
       </c>
     </row>
@@ -14290,15 +14292,15 @@
       <c r="D12" s="15" t="n"/>
       <c r="E12" s="15" t="n"/>
       <c r="F12" s="22">
-        <f>IF(E12=0,0,MIN(1,C12/E12))</f>
+        <f>IF(A12="","",IF(E12=0,0,MIN(1,C12/E12)))</f>
         <v/>
       </c>
       <c r="G12" s="20">
-        <f>IF(E12=0,0,MAX(0,E12-C12))</f>
+        <f>IF(A12="","",IF(E12=0,0,MAX(0,E12-C12)))</f>
         <v/>
       </c>
       <c r="H12" s="31">
-        <f>IF(OR(D12=0,G12&lt;=0),"N/A",ROUNDUP(G12/D12,0))</f>
+        <f>IF(A12="","",IF(OR(D12=0,G12&lt;=0),"N/A",ROUNDUP(G12/D12,0)))</f>
         <v/>
       </c>
     </row>
@@ -14309,15 +14311,15 @@
       <c r="D13" s="15" t="n"/>
       <c r="E13" s="15" t="n"/>
       <c r="F13" s="22">
-        <f>IF(E13=0,0,MIN(1,C13/E13))</f>
+        <f>IF(A13="","",IF(E13=0,0,MIN(1,C13/E13)))</f>
         <v/>
       </c>
       <c r="G13" s="20">
-        <f>IF(E13=0,0,MAX(0,E13-C13))</f>
+        <f>IF(A13="","",IF(E13=0,0,MAX(0,E13-C13)))</f>
         <v/>
       </c>
       <c r="H13" s="31">
-        <f>IF(OR(D13=0,G13&lt;=0),"N/A",ROUNDUP(G13/D13,0))</f>
+        <f>IF(A13="","",IF(OR(D13=0,G13&lt;=0),"N/A",ROUNDUP(G13/D13,0)))</f>
         <v/>
       </c>
     </row>
@@ -14328,15 +14330,15 @@
       <c r="D14" s="15" t="n"/>
       <c r="E14" s="15" t="n"/>
       <c r="F14" s="22">
-        <f>IF(E14=0,0,MIN(1,C14/E14))</f>
+        <f>IF(A14="","",IF(E14=0,0,MIN(1,C14/E14)))</f>
         <v/>
       </c>
       <c r="G14" s="20">
-        <f>IF(E14=0,0,MAX(0,E14-C14))</f>
+        <f>IF(A14="","",IF(E14=0,0,MAX(0,E14-C14)))</f>
         <v/>
       </c>
       <c r="H14" s="31">
-        <f>IF(OR(D14=0,G14&lt;=0),"N/A",ROUNDUP(G14/D14,0))</f>
+        <f>IF(A14="","",IF(OR(D14=0,G14&lt;=0),"N/A",ROUNDUP(G14/D14,0)))</f>
         <v/>
       </c>
     </row>
@@ -14347,15 +14349,15 @@
       <c r="D15" s="15" t="n"/>
       <c r="E15" s="15" t="n"/>
       <c r="F15" s="22">
-        <f>IF(E15=0,0,MIN(1,C15/E15))</f>
+        <f>IF(A15="","",IF(E15=0,0,MIN(1,C15/E15)))</f>
         <v/>
       </c>
       <c r="G15" s="20">
-        <f>IF(E15=0,0,MAX(0,E15-C15))</f>
+        <f>IF(A15="","",IF(E15=0,0,MAX(0,E15-C15)))</f>
         <v/>
       </c>
       <c r="H15" s="31">
-        <f>IF(OR(D15=0,G15&lt;=0),"N/A",ROUNDUP(G15/D15,0))</f>
+        <f>IF(A15="","",IF(OR(D15=0,G15&lt;=0),"N/A",ROUNDUP(G15/D15,0)))</f>
         <v/>
       </c>
     </row>
@@ -14366,15 +14368,15 @@
       <c r="D16" s="15" t="n"/>
       <c r="E16" s="15" t="n"/>
       <c r="F16" s="22">
-        <f>IF(E16=0,0,MIN(1,C16/E16))</f>
+        <f>IF(A16="","",IF(E16=0,0,MIN(1,C16/E16)))</f>
         <v/>
       </c>
       <c r="G16" s="20">
-        <f>IF(E16=0,0,MAX(0,E16-C16))</f>
+        <f>IF(A16="","",IF(E16=0,0,MAX(0,E16-C16)))</f>
         <v/>
       </c>
       <c r="H16" s="31">
-        <f>IF(OR(D16=0,G16&lt;=0),"N/A",ROUNDUP(G16/D16,0))</f>
+        <f>IF(A16="","",IF(OR(D16=0,G16&lt;=0),"N/A",ROUNDUP(G16/D16,0)))</f>
         <v/>
       </c>
     </row>
@@ -14385,15 +14387,15 @@
       <c r="D17" s="15" t="n"/>
       <c r="E17" s="15" t="n"/>
       <c r="F17" s="22">
-        <f>IF(E17=0,0,MIN(1,C17/E17))</f>
+        <f>IF(A17="","",IF(E17=0,0,MIN(1,C17/E17)))</f>
         <v/>
       </c>
       <c r="G17" s="20">
-        <f>IF(E17=0,0,MAX(0,E17-C17))</f>
+        <f>IF(A17="","",IF(E17=0,0,MAX(0,E17-C17)))</f>
         <v/>
       </c>
       <c r="H17" s="31">
-        <f>IF(OR(D17=0,G17&lt;=0),"N/A",ROUNDUP(G17/D17,0))</f>
+        <f>IF(A17="","",IF(OR(D17=0,G17&lt;=0),"N/A",ROUNDUP(G17/D17,0)))</f>
         <v/>
       </c>
     </row>
@@ -14404,15 +14406,15 @@
       <c r="D18" s="15" t="n"/>
       <c r="E18" s="15" t="n"/>
       <c r="F18" s="22">
-        <f>IF(E18=0,0,MIN(1,C18/E18))</f>
+        <f>IF(A18="","",IF(E18=0,0,MIN(1,C18/E18)))</f>
         <v/>
       </c>
       <c r="G18" s="20">
-        <f>IF(E18=0,0,MAX(0,E18-C18))</f>
+        <f>IF(A18="","",IF(E18=0,0,MAX(0,E18-C18)))</f>
         <v/>
       </c>
       <c r="H18" s="31">
-        <f>IF(OR(D18=0,G18&lt;=0),"N/A",ROUNDUP(G18/D18,0))</f>
+        <f>IF(A18="","",IF(OR(D18=0,G18&lt;=0),"N/A",ROUNDUP(G18/D18,0)))</f>
         <v/>
       </c>
     </row>
@@ -14423,15 +14425,15 @@
       <c r="D19" s="15" t="n"/>
       <c r="E19" s="15" t="n"/>
       <c r="F19" s="22">
-        <f>IF(E19=0,0,MIN(1,C19/E19))</f>
+        <f>IF(A19="","",IF(E19=0,0,MIN(1,C19/E19)))</f>
         <v/>
       </c>
       <c r="G19" s="20">
-        <f>IF(E19=0,0,MAX(0,E19-C19))</f>
+        <f>IF(A19="","",IF(E19=0,0,MAX(0,E19-C19)))</f>
         <v/>
       </c>
       <c r="H19" s="31">
-        <f>IF(OR(D19=0,G19&lt;=0),"N/A",ROUNDUP(G19/D19,0))</f>
+        <f>IF(A19="","",IF(OR(D19=0,G19&lt;=0),"N/A",ROUNDUP(G19/D19,0)))</f>
         <v/>
       </c>
     </row>
@@ -14442,15 +14444,15 @@
       <c r="D20" s="15" t="n"/>
       <c r="E20" s="15" t="n"/>
       <c r="F20" s="22">
-        <f>IF(E20=0,0,MIN(1,C20/E20))</f>
+        <f>IF(A20="","",IF(E20=0,0,MIN(1,C20/E20)))</f>
         <v/>
       </c>
       <c r="G20" s="20">
-        <f>IF(E20=0,0,MAX(0,E20-C20))</f>
+        <f>IF(A20="","",IF(E20=0,0,MAX(0,E20-C20)))</f>
         <v/>
       </c>
       <c r="H20" s="31">
-        <f>IF(OR(D20=0,G20&lt;=0),"N/A",ROUNDUP(G20/D20,0))</f>
+        <f>IF(A20="","",IF(OR(D20=0,G20&lt;=0),"N/A",ROUNDUP(G20/D20,0)))</f>
         <v/>
       </c>
     </row>
@@ -14461,15 +14463,15 @@
       <c r="D21" s="15" t="n"/>
       <c r="E21" s="15" t="n"/>
       <c r="F21" s="22">
-        <f>IF(E21=0,0,MIN(1,C21/E21))</f>
+        <f>IF(A21="","",IF(E21=0,0,MIN(1,C21/E21)))</f>
         <v/>
       </c>
       <c r="G21" s="20">
-        <f>IF(E21=0,0,MAX(0,E21-C21))</f>
+        <f>IF(A21="","",IF(E21=0,0,MAX(0,E21-C21)))</f>
         <v/>
       </c>
       <c r="H21" s="31">
-        <f>IF(OR(D21=0,G21&lt;=0),"N/A",ROUNDUP(G21/D21,0))</f>
+        <f>IF(A21="","",IF(OR(D21=0,G21&lt;=0),"N/A",ROUNDUP(G21/D21,0)))</f>
         <v/>
       </c>
     </row>
@@ -14480,15 +14482,15 @@
       <c r="D22" s="15" t="n"/>
       <c r="E22" s="15" t="n"/>
       <c r="F22" s="22">
-        <f>IF(E22=0,0,MIN(1,C22/E22))</f>
+        <f>IF(A22="","",IF(E22=0,0,MIN(1,C22/E22)))</f>
         <v/>
       </c>
       <c r="G22" s="20">
-        <f>IF(E22=0,0,MAX(0,E22-C22))</f>
+        <f>IF(A22="","",IF(E22=0,0,MAX(0,E22-C22)))</f>
         <v/>
       </c>
       <c r="H22" s="31">
-        <f>IF(OR(D22=0,G22&lt;=0),"N/A",ROUNDUP(G22/D22,0))</f>
+        <f>IF(A22="","",IF(OR(D22=0,G22&lt;=0),"N/A",ROUNDUP(G22/D22,0)))</f>
         <v/>
       </c>
     </row>
@@ -14499,15 +14501,15 @@
       <c r="D23" s="15" t="n"/>
       <c r="E23" s="15" t="n"/>
       <c r="F23" s="22">
-        <f>IF(E23=0,0,MIN(1,C23/E23))</f>
+        <f>IF(A23="","",IF(E23=0,0,MIN(1,C23/E23)))</f>
         <v/>
       </c>
       <c r="G23" s="20">
-        <f>IF(E23=0,0,MAX(0,E23-C23))</f>
+        <f>IF(A23="","",IF(E23=0,0,MAX(0,E23-C23)))</f>
         <v/>
       </c>
       <c r="H23" s="31">
-        <f>IF(OR(D23=0,G23&lt;=0),"N/A",ROUNDUP(G23/D23,0))</f>
+        <f>IF(A23="","",IF(OR(D23=0,G23&lt;=0),"N/A",ROUNDUP(G23/D23,0)))</f>
         <v/>
       </c>
     </row>
@@ -14518,15 +14520,15 @@
       <c r="D24" s="15" t="n"/>
       <c r="E24" s="15" t="n"/>
       <c r="F24" s="22">
-        <f>IF(E24=0,0,MIN(1,C24/E24))</f>
+        <f>IF(A24="","",IF(E24=0,0,MIN(1,C24/E24)))</f>
         <v/>
       </c>
       <c r="G24" s="20">
-        <f>IF(E24=0,0,MAX(0,E24-C24))</f>
+        <f>IF(A24="","",IF(E24=0,0,MAX(0,E24-C24)))</f>
         <v/>
       </c>
       <c r="H24" s="31">
-        <f>IF(OR(D24=0,G24&lt;=0),"N/A",ROUNDUP(G24/D24,0))</f>
+        <f>IF(A24="","",IF(OR(D24=0,G24&lt;=0),"N/A",ROUNDUP(G24/D24,0)))</f>
         <v/>
       </c>
     </row>
@@ -14662,11 +14664,11 @@
       <c r="E5" s="15" t="n"/>
       <c r="F5" s="25" t="n"/>
       <c r="G5" s="20">
-        <f>IF(C5=0,0,D5-C5)</f>
+        <f>IF(A5="","",IF(C5=0,0,D5-C5))</f>
         <v/>
       </c>
       <c r="H5" s="22">
-        <f>IF(C5=0,0,G5/C5)</f>
+        <f>IF(A5="","",IF(C5=0,0,G5/C5))</f>
         <v/>
       </c>
       <c r="I5" s="33" t="n"/>
@@ -14679,11 +14681,11 @@
       <c r="E6" s="15" t="n"/>
       <c r="F6" s="25" t="n"/>
       <c r="G6" s="20">
-        <f>IF(C6=0,0,D6-C6)</f>
+        <f>IF(A6="","",IF(C6=0,0,D6-C6))</f>
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>IF(C6=0,0,G6/C6)</f>
+        <f>IF(A6="","",IF(C6=0,0,G6/C6))</f>
         <v/>
       </c>
       <c r="I6" s="33" t="n"/>
@@ -14696,11 +14698,11 @@
       <c r="E7" s="15" t="n"/>
       <c r="F7" s="25" t="n"/>
       <c r="G7" s="20">
-        <f>IF(C7=0,0,D7-C7)</f>
+        <f>IF(A7="","",IF(C7=0,0,D7-C7))</f>
         <v/>
       </c>
       <c r="H7" s="22">
-        <f>IF(C7=0,0,G7/C7)</f>
+        <f>IF(A7="","",IF(C7=0,0,G7/C7))</f>
         <v/>
       </c>
       <c r="I7" s="33" t="n"/>
@@ -14713,11 +14715,11 @@
       <c r="E8" s="15" t="n"/>
       <c r="F8" s="25" t="n"/>
       <c r="G8" s="20">
-        <f>IF(C8=0,0,D8-C8)</f>
+        <f>IF(A8="","",IF(C8=0,0,D8-C8))</f>
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>IF(C8=0,0,G8/C8)</f>
+        <f>IF(A8="","",IF(C8=0,0,G8/C8))</f>
         <v/>
       </c>
       <c r="I8" s="33" t="n"/>
@@ -14730,11 +14732,11 @@
       <c r="E9" s="15" t="n"/>
       <c r="F9" s="25" t="n"/>
       <c r="G9" s="20">
-        <f>IF(C9=0,0,D9-C9)</f>
+        <f>IF(A9="","",IF(C9=0,0,D9-C9))</f>
         <v/>
       </c>
       <c r="H9" s="22">
-        <f>IF(C9=0,0,G9/C9)</f>
+        <f>IF(A9="","",IF(C9=0,0,G9/C9))</f>
         <v/>
       </c>
       <c r="I9" s="33" t="n"/>
@@ -14747,11 +14749,11 @@
       <c r="E10" s="15" t="n"/>
       <c r="F10" s="25" t="n"/>
       <c r="G10" s="20">
-        <f>IF(C10=0,0,D10-C10)</f>
+        <f>IF(A10="","",IF(C10=0,0,D10-C10))</f>
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>IF(C10=0,0,G10/C10)</f>
+        <f>IF(A10="","",IF(C10=0,0,G10/C10))</f>
         <v/>
       </c>
       <c r="I10" s="33" t="n"/>
@@ -14764,11 +14766,11 @@
       <c r="E11" s="15" t="n"/>
       <c r="F11" s="25" t="n"/>
       <c r="G11" s="20">
-        <f>IF(C11=0,0,D11-C11)</f>
+        <f>IF(A11="","",IF(C11=0,0,D11-C11))</f>
         <v/>
       </c>
       <c r="H11" s="22">
-        <f>IF(C11=0,0,G11/C11)</f>
+        <f>IF(A11="","",IF(C11=0,0,G11/C11))</f>
         <v/>
       </c>
       <c r="I11" s="33" t="n"/>
@@ -14781,11 +14783,11 @@
       <c r="E12" s="15" t="n"/>
       <c r="F12" s="25" t="n"/>
       <c r="G12" s="20">
-        <f>IF(C12=0,0,D12-C12)</f>
+        <f>IF(A12="","",IF(C12=0,0,D12-C12))</f>
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>IF(C12=0,0,G12/C12)</f>
+        <f>IF(A12="","",IF(C12=0,0,G12/C12))</f>
         <v/>
       </c>
       <c r="I12" s="33" t="n"/>
@@ -14798,11 +14800,11 @@
       <c r="E13" s="15" t="n"/>
       <c r="F13" s="25" t="n"/>
       <c r="G13" s="20">
-        <f>IF(C13=0,0,D13-C13)</f>
+        <f>IF(A13="","",IF(C13=0,0,D13-C13))</f>
         <v/>
       </c>
       <c r="H13" s="22">
-        <f>IF(C13=0,0,G13/C13)</f>
+        <f>IF(A13="","",IF(C13=0,0,G13/C13))</f>
         <v/>
       </c>
       <c r="I13" s="33" t="n"/>
@@ -14815,11 +14817,11 @@
       <c r="E14" s="15" t="n"/>
       <c r="F14" s="25" t="n"/>
       <c r="G14" s="20">
-        <f>IF(C14=0,0,D14-C14)</f>
+        <f>IF(A14="","",IF(C14=0,0,D14-C14))</f>
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>IF(C14=0,0,G14/C14)</f>
+        <f>IF(A14="","",IF(C14=0,0,G14/C14))</f>
         <v/>
       </c>
       <c r="I14" s="33" t="n"/>
@@ -14832,11 +14834,11 @@
       <c r="E15" s="15" t="n"/>
       <c r="F15" s="25" t="n"/>
       <c r="G15" s="20">
-        <f>IF(C15=0,0,D15-C15)</f>
+        <f>IF(A15="","",IF(C15=0,0,D15-C15))</f>
         <v/>
       </c>
       <c r="H15" s="22">
-        <f>IF(C15=0,0,G15/C15)</f>
+        <f>IF(A15="","",IF(C15=0,0,G15/C15))</f>
         <v/>
       </c>
       <c r="I15" s="33" t="n"/>
@@ -14849,11 +14851,11 @@
       <c r="E16" s="15" t="n"/>
       <c r="F16" s="25" t="n"/>
       <c r="G16" s="20">
-        <f>IF(C16=0,0,D16-C16)</f>
+        <f>IF(A16="","",IF(C16=0,0,D16-C16))</f>
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>IF(C16=0,0,G16/C16)</f>
+        <f>IF(A16="","",IF(C16=0,0,G16/C16))</f>
         <v/>
       </c>
       <c r="I16" s="33" t="n"/>
@@ -14866,11 +14868,11 @@
       <c r="E17" s="15" t="n"/>
       <c r="F17" s="25" t="n"/>
       <c r="G17" s="20">
-        <f>IF(C17=0,0,D17-C17)</f>
+        <f>IF(A17="","",IF(C17=0,0,D17-C17))</f>
         <v/>
       </c>
       <c r="H17" s="22">
-        <f>IF(C17=0,0,G17/C17)</f>
+        <f>IF(A17="","",IF(C17=0,0,G17/C17))</f>
         <v/>
       </c>
       <c r="I17" s="33" t="n"/>
@@ -14883,11 +14885,11 @@
       <c r="E18" s="15" t="n"/>
       <c r="F18" s="25" t="n"/>
       <c r="G18" s="20">
-        <f>IF(C18=0,0,D18-C18)</f>
+        <f>IF(A18="","",IF(C18=0,0,D18-C18))</f>
         <v/>
       </c>
       <c r="H18" s="22">
-        <f>IF(C18=0,0,G18/C18)</f>
+        <f>IF(A18="","",IF(C18=0,0,G18/C18))</f>
         <v/>
       </c>
       <c r="I18" s="33" t="n"/>
@@ -14900,11 +14902,11 @@
       <c r="E19" s="15" t="n"/>
       <c r="F19" s="25" t="n"/>
       <c r="G19" s="20">
-        <f>IF(C19=0,0,D19-C19)</f>
+        <f>IF(A19="","",IF(C19=0,0,D19-C19))</f>
         <v/>
       </c>
       <c r="H19" s="22">
-        <f>IF(C19=0,0,G19/C19)</f>
+        <f>IF(A19="","",IF(C19=0,0,G19/C19))</f>
         <v/>
       </c>
       <c r="I19" s="33" t="n"/>
@@ -14917,11 +14919,11 @@
       <c r="E20" s="15" t="n"/>
       <c r="F20" s="25" t="n"/>
       <c r="G20" s="20">
-        <f>IF(C20=0,0,D20-C20)</f>
+        <f>IF(A20="","",IF(C20=0,0,D20-C20))</f>
         <v/>
       </c>
       <c r="H20" s="22">
-        <f>IF(C20=0,0,G20/C20)</f>
+        <f>IF(A20="","",IF(C20=0,0,G20/C20))</f>
         <v/>
       </c>
       <c r="I20" s="33" t="n"/>
@@ -14934,11 +14936,11 @@
       <c r="E21" s="15" t="n"/>
       <c r="F21" s="25" t="n"/>
       <c r="G21" s="20">
-        <f>IF(C21=0,0,D21-C21)</f>
+        <f>IF(A21="","",IF(C21=0,0,D21-C21))</f>
         <v/>
       </c>
       <c r="H21" s="22">
-        <f>IF(C21=0,0,G21/C21)</f>
+        <f>IF(A21="","",IF(C21=0,0,G21/C21))</f>
         <v/>
       </c>
       <c r="I21" s="33" t="n"/>
@@ -14951,11 +14953,11 @@
       <c r="E22" s="15" t="n"/>
       <c r="F22" s="25" t="n"/>
       <c r="G22" s="20">
-        <f>IF(C22=0,0,D22-C22)</f>
+        <f>IF(A22="","",IF(C22=0,0,D22-C22))</f>
         <v/>
       </c>
       <c r="H22" s="22">
-        <f>IF(C22=0,0,G22/C22)</f>
+        <f>IF(A22="","",IF(C22=0,0,G22/C22))</f>
         <v/>
       </c>
       <c r="I22" s="33" t="n"/>
@@ -14968,11 +14970,11 @@
       <c r="E23" s="15" t="n"/>
       <c r="F23" s="25" t="n"/>
       <c r="G23" s="20">
-        <f>IF(C23=0,0,D23-C23)</f>
+        <f>IF(A23="","",IF(C23=0,0,D23-C23))</f>
         <v/>
       </c>
       <c r="H23" s="22">
-        <f>IF(C23=0,0,G23/C23)</f>
+        <f>IF(A23="","",IF(C23=0,0,G23/C23))</f>
         <v/>
       </c>
       <c r="I23" s="33" t="n"/>
@@ -14985,11 +14987,11 @@
       <c r="E24" s="15" t="n"/>
       <c r="F24" s="25" t="n"/>
       <c r="G24" s="20">
-        <f>IF(C24=0,0,D24-C24)</f>
+        <f>IF(A24="","",IF(C24=0,0,D24-C24))</f>
         <v/>
       </c>
       <c r="H24" s="22">
-        <f>IF(C24=0,0,G24/C24)</f>
+        <f>IF(A24="","",IF(C24=0,0,G24/C24))</f>
         <v/>
       </c>
       <c r="I24" s="33" t="n"/>

</xml_diff>